<commit_message>
Checkpoint dataset, benchmark, and optimization prompt updates
</commit_message>
<xml_diff>
--- a/apps/web/fixtures/demo-workbooks/retailer-transactions-demo-query-logs.xlsx
+++ b/apps/web/fixtures/demo-workbooks/retailer-transactions-demo-query-logs.xlsx
@@ -4,7 +4,6 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="query_logs" sheetId="1" r:id="rId1"/>
-    <sheet name="notes" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -479,9 +478,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-01-01')
   AND business_date &lt;= DATE('2025-01-07')
@@ -502,7 +501,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K2" t="str">
-        <v>Show daily units sold, revenue, and cost across all stores for SKU-00001, SKU-00007, SKU-00013 from 2025-01-01 to 2025-01-07.</v>
+        <v>Show daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) across all stores for SKU-00001, SKU-00007, SKU-00013 from 2025-01-01 to 2025-01-07. Exclude returned rows.</v>
       </c>
       <c r="L2" t="str">
         <v>query_log_rollup_01</v>
@@ -573,9 +572,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-01-01')
     AND business_date &lt;= DATE('2025-01-07')
@@ -606,7 +605,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K3" t="str">
-        <v>Show the same daily SKU metrics across all stores for SKU-00001, SKU-00007, SKU-00013 from 2025-01-01 to 2025-01-07, but include zero rows for days with no sales.</v>
+        <v>Show the same daily SKU metrics across all stores for SKU-00001, SKU-00007, SKU-00013 from 2025-01-01 to 2025-01-07, but include zero rows for days with no sales. Exclude returned rows.</v>
       </c>
       <c r="L3" t="str">
         <v>query_log_zero_fill_01</v>
@@ -653,9 +652,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-01-08')
   AND business_date &lt;= DATE('2025-01-14')
@@ -676,7 +675,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K4" t="str">
-        <v>Give me a day-by-day sales view for SKU-00022, SKU-00027, SKU-00031 between 2025-01-08 and 2025-01-14, including units, revenue, and cost for the whole business.</v>
+        <v>Give me a day-by-day sales view for SKU-00022, SKU-00027, SKU-00031 between 2025-01-08 and 2025-01-14, including units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for the whole business. Exclude returned rows.</v>
       </c>
       <c r="L4" t="str">
         <v>query_log_rollup_02</v>
@@ -747,9 +746,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-01-08')
     AND business_date &lt;= DATE('2025-01-14')
@@ -780,7 +779,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K5" t="str">
-        <v>Give me the daily SKU trend for SKU-00022, SKU-00027, SKU-00031 between 2025-01-08 and 2025-01-14, and backfill missing dates with zeroes when nothing sold.</v>
+        <v>Give me the daily SKU trend for SKU-00022, SKU-00027, SKU-00031 between 2025-01-08 and 2025-01-14, and backfill missing dates with zeroes when nothing sold. Exclude returned rows.</v>
       </c>
       <c r="L5" t="str">
         <v>query_log_zero_fill_02</v>
@@ -827,9 +826,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-01-15')
   AND business_date &lt;= DATE('2025-01-21')
@@ -850,7 +849,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K6" t="str">
-        <v>I want the daily SKU totals for SKU-00044, SKU-00048, SKU-00053 over 2025-01-15 to 2025-01-21 with units sold, revenue, and cost rolled up across every store.</v>
+        <v>I want the daily SKU totals for SKU-00044, SKU-00048, SKU-00053 over 2025-01-15 to 2025-01-21 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) rolled up across every store. Exclude returned rows.</v>
       </c>
       <c r="L6" t="str">
         <v>query_log_rollup_03</v>
@@ -921,9 +920,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-01-15')
     AND business_date &lt;= DATE('2025-01-21')
@@ -954,7 +953,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K7" t="str">
-        <v>I need a complete SKU-by-day series for SKU-00044, SKU-00048, SKU-00053 from 2025-01-15 to 2025-01-21, with units, revenue, and cost set to 0 on no-sale days.</v>
+        <v>I need a complete SKU-by-day series for SKU-00044, SKU-00048, SKU-00053 from 2025-01-15 to 2025-01-21, with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) set to 0 on no-sale days. Exclude returned rows.</v>
       </c>
       <c r="L7" t="str">
         <v>query_log_zero_fill_03</v>
@@ -1001,9 +1000,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-01-22')
   AND business_date &lt;= DATE('2025-01-31')
@@ -1024,7 +1023,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K8" t="str">
-        <v>Can you break out daily units, revenue, and cost for SKU-00061, SKU-00064, SKU-00069 from 2025-01-22 through 2025-01-31, summed across all stores?</v>
+        <v>Can you break out daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for SKU-00061, SKU-00064, SKU-00069 from 2025-01-22 through 2025-01-31, summed across all stores? Exclude returned rows.</v>
       </c>
       <c r="L8" t="str">
         <v>query_log_rollup_04</v>
@@ -1095,9 +1094,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-01-22')
     AND business_date &lt;= DATE('2025-01-31')
@@ -1128,7 +1127,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K9" t="str">
-        <v>Return the daily all-store metrics for SKU-00061, SKU-00064, SKU-00069 over 2025-01-22 to 2025-01-31, making sure dates with no sales still appear as zeroes.</v>
+        <v>Return the daily all-store metrics for SKU-00061, SKU-00064, SKU-00069 over 2025-01-22 to 2025-01-31, making sure dates with no sales still appear as zeroes. Exclude returned rows.</v>
       </c>
       <c r="L9" t="str">
         <v>query_log_zero_fill_04</v>
@@ -1175,9 +1174,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-02-01')
   AND business_date &lt;= DATE('2025-02-07')
@@ -1198,7 +1197,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K10" t="str">
-        <v>Pull a daily all-store SKU summary for SKU-00078, SKU-00082, SKU-00086 between 2025-02-01 and 2025-02-07 with units sold, revenue, and cost.</v>
+        <v>Pull a daily all-store SKU summary for SKU-00078, SKU-00082, SKU-00086 between 2025-02-01 and 2025-02-07 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT). Exclude returned rows.</v>
       </c>
       <c r="L10" t="str">
         <v>query_log_rollup_05</v>
@@ -1269,9 +1268,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-02-01')
     AND business_date &lt;= DATE('2025-02-07')
@@ -1302,7 +1301,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K11" t="str">
-        <v>Build the same daily rollup for SKU-00078, SKU-00082, SKU-00086 from 2025-02-01 through 2025-02-07, but don’t drop empty days; fill them with 0s instead.</v>
+        <v>Build the same daily rollup for SKU-00078, SKU-00082, SKU-00086 from 2025-02-01 through 2025-02-07, but don’t drop empty days; fill them with 0s instead. Exclude returned rows.</v>
       </c>
       <c r="L11" t="str">
         <v>query_log_zero_fill_05</v>
@@ -1349,9 +1348,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-02-08')
   AND business_date &lt;= DATE('2025-02-14')
@@ -1372,7 +1371,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K12" t="str">
-        <v>Show daily units sold, revenue, and cost across all stores for SKU-00094, SKU-00099, SKU-00104 from 2025-02-08 to 2025-02-14.</v>
+        <v>Show daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) across all stores for SKU-00094, SKU-00099, SKU-00104 from 2025-02-08 to 2025-02-14. Exclude returned rows.</v>
       </c>
       <c r="L12" t="str">
         <v>query_log_rollup_06</v>
@@ -1443,9 +1442,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-02-08')
     AND business_date &lt;= DATE('2025-02-14')
@@ -1476,7 +1475,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K13" t="str">
-        <v>Show the same daily SKU metrics across all stores for SKU-00094, SKU-00099, SKU-00104 from 2025-02-08 to 2025-02-14, but include zero rows for days with no sales.</v>
+        <v>Show the same daily SKU metrics across all stores for SKU-00094, SKU-00099, SKU-00104 from 2025-02-08 to 2025-02-14, but include zero rows for days with no sales. Exclude returned rows.</v>
       </c>
       <c r="L13" t="str">
         <v>query_log_zero_fill_06</v>
@@ -1523,9 +1522,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-02-15')
   AND business_date &lt;= DATE('2025-02-21')
@@ -1546,7 +1545,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K14" t="str">
-        <v>Give me a day-by-day sales view for SKU-00111, SKU-00115, SKU-00119 between 2025-02-15 and 2025-02-21, including units, revenue, and cost for the whole business.</v>
+        <v>Give me a day-by-day sales view for SKU-00111, SKU-00115, SKU-00119 between 2025-02-15 and 2025-02-21, including units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for the whole business. Exclude returned rows.</v>
       </c>
       <c r="L14" t="str">
         <v>query_log_rollup_07</v>
@@ -1617,9 +1616,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-02-15')
     AND business_date &lt;= DATE('2025-02-21')
@@ -1650,7 +1649,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K15" t="str">
-        <v>Give me the daily SKU trend for SKU-00111, SKU-00115, SKU-00119 between 2025-02-15 and 2025-02-21, and backfill missing dates with zeroes when nothing sold.</v>
+        <v>Give me the daily SKU trend for SKU-00111, SKU-00115, SKU-00119 between 2025-02-15 and 2025-02-21, and backfill missing dates with zeroes when nothing sold. Exclude returned rows.</v>
       </c>
       <c r="L15" t="str">
         <v>query_log_zero_fill_07</v>
@@ -1697,9 +1696,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-02-22')
   AND business_date &lt;= DATE('2025-02-28')
@@ -1720,7 +1719,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K16" t="str">
-        <v>I want the daily SKU totals for SKU-00127, SKU-00132, SKU-00137 over 2025-02-22 to 2025-02-28 with units sold, revenue, and cost rolled up across every store.</v>
+        <v>I want the daily SKU totals for SKU-00127, SKU-00132, SKU-00137 over 2025-02-22 to 2025-02-28 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) rolled up across every store. Exclude returned rows.</v>
       </c>
       <c r="L16" t="str">
         <v>query_log_rollup_08</v>
@@ -1791,9 +1790,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-02-22')
     AND business_date &lt;= DATE('2025-02-28')
@@ -1824,7 +1823,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K17" t="str">
-        <v>I need a complete SKU-by-day series for SKU-00127, SKU-00132, SKU-00137 from 2025-02-22 to 2025-02-28, with units, revenue, and cost set to 0 on no-sale days.</v>
+        <v>I need a complete SKU-by-day series for SKU-00127, SKU-00132, SKU-00137 from 2025-02-22 to 2025-02-28, with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) set to 0 on no-sale days. Exclude returned rows.</v>
       </c>
       <c r="L17" t="str">
         <v>query_log_zero_fill_08</v>
@@ -1871,9 +1870,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-03-01')
   AND business_date &lt;= DATE('2025-03-15')
@@ -1894,7 +1893,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K18" t="str">
-        <v>Can you break out daily units, revenue, and cost for SKU-00146, SKU-00152, SKU-00158 from 2025-03-01 through 2025-03-15, summed across all stores?</v>
+        <v>Can you break out daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for SKU-00146, SKU-00152, SKU-00158 from 2025-03-01 through 2025-03-15, summed across all stores? Exclude returned rows.</v>
       </c>
       <c r="L18" t="str">
         <v>query_log_rollup_09</v>
@@ -1965,9 +1964,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-03-01')
     AND business_date &lt;= DATE('2025-03-15')
@@ -1998,7 +1997,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K19" t="str">
-        <v>Return the daily all-store metrics for SKU-00146, SKU-00152, SKU-00158 over 2025-03-01 to 2025-03-15, making sure dates with no sales still appear as zeroes.</v>
+        <v>Return the daily all-store metrics for SKU-00146, SKU-00152, SKU-00158 over 2025-03-01 to 2025-03-15, making sure dates with no sales still appear as zeroes. Exclude returned rows.</v>
       </c>
       <c r="L19" t="str">
         <v>query_log_zero_fill_09</v>
@@ -2045,9 +2044,9 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(units) AS units_sold,
-  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-  SUM(cogs_ex_vat) AS cost_ex_vat
+  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
 FROM clean_transactions
 WHERE business_date &gt;= DATE('2025-03-16')
   AND business_date &lt;= DATE('2025-03-31')
@@ -2068,7 +2067,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K20" t="str">
-        <v>Pull a daily all-store SKU summary for SKU-00163, SKU-00169, SKU-00175 between 2025-03-16 and 2025-03-31 with units sold, revenue, and cost.</v>
+        <v>Pull a daily all-store SKU summary for SKU-00163, SKU-00169, SKU-00175 between 2025-03-16 and 2025-03-31 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT). Exclude returned rows.</v>
       </c>
       <c r="L20" t="str">
         <v>query_log_rollup_10</v>
@@ -2139,9 +2138,9 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(units) AS units_sold,
-    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
-    SUM(cogs_ex_vat) AS cost_ex_vat
+    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
+    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
+    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
   FROM clean_transactions
   WHERE business_date &gt;= DATE('2025-03-16')
     AND business_date &lt;= DATE('2025-03-31')
@@ -2172,7 +2171,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K21" t="str">
-        <v>Build the same daily rollup for SKU-00163, SKU-00169, SKU-00175 from 2025-03-16 through 2025-03-31, but don’t drop empty days; fill them with 0s instead.</v>
+        <v>Build the same daily rollup for SKU-00163, SKU-00169, SKU-00175 from 2025-03-16 through 2025-03-31, but don’t drop empty days; fill them with 0s instead. Exclude returned rows.</v>
       </c>
       <c r="L21" t="str">
         <v>query_log_zero_fill_10</v>
@@ -2204,47 +2203,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:S21"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>assumption</v>
-      </c>
-      <c r="B1" t="str">
-        <v>detail</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>SQL assumes a cleaned fact table named clean_transactions with snake_case columns derived from the demo workbook.</v>
-      </c>
-      <c r="B2" t="str">
-        <v>This fixture is meant to seed query-log history, not to assert the exact pipeline output from a specific import run.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>patternType=sku_daily_rollup</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Daily grouped sales by SKU and business_date across all stores, with units_sold, revenue_incl_vat, and cost_ex_vat.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>patternType=sku_daily_rollup_zero_fill</v>
-      </c>
-      <c r="B4" t="str">
-        <v>A date spine plus grouped sales so missing SKU-day combinations return zero values instead of disappearing.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Improve optimization loop, parity checks, and benchmark/eval tooling
</commit_message>
<xml_diff>
--- a/apps/web/fixtures/demo-workbooks/retailer-transactions-demo-query-logs.xlsx
+++ b/apps/web/fixtures/demo-workbooks/retailer-transactions-demo-query-logs.xlsx
@@ -478,13 +478,14 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
 WHERE business_date &gt;= DATE('2025-01-01')
   AND business_date &lt;= DATE('2025-01-07')
   AND item_sku IN ('SKU-00001', 'SKU-00007', 'SKU-00013')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
 GROUP BY item_sku, business_date
 ORDER BY item_sku, business_date;</v>
       </c>
@@ -501,7 +502,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K2" t="str">
-        <v>Show daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) across all stores for SKU-00001, SKU-00007, SKU-00013 from 2025-01-01 to 2025-01-07. Exclude returned rows.</v>
+        <v>Show daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) across all stores for SKU-00001, SKU-00007, SKU-00013 from 2025-01-01 to 2025-01-07. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L2" t="str">
         <v>query_log_rollup_01</v>
@@ -510,7 +511,7 @@
         <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
       </c>
       <c r="N2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O2" t="str">
         <v>dataset_retailer_transactions_demo</v>
@@ -549,7 +550,7 @@
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-01-01')
     AND business_date &lt;= DATE('2025-01-07')
 ),
@@ -572,13 +573,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-01-01')
     AND business_date &lt;= DATE('2025-01-07')
     AND item_sku IN ('SKU-00001', 'SKU-00007', 'SKU-00013')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -605,7 +607,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K3" t="str">
-        <v>Show the same daily SKU metrics across all stores for SKU-00001, SKU-00007, SKU-00013 from 2025-01-01 to 2025-01-07, but include zero rows for days with no sales. Exclude returned rows.</v>
+        <v>Show the same daily SKU metrics across all stores for SKU-00001, SKU-00007, SKU-00013 from 2025-01-01 to 2025-01-07, but include zero rows for days with no sales. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L3" t="str">
         <v>query_log_zero_fill_01</v>
@@ -652,13 +654,14 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
 WHERE business_date &gt;= DATE('2025-01-08')
   AND business_date &lt;= DATE('2025-01-14')
   AND item_sku IN ('SKU-00022', 'SKU-00027', 'SKU-00031')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
 GROUP BY item_sku, business_date
 ORDER BY item_sku, business_date;</v>
       </c>
@@ -675,7 +678,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K4" t="str">
-        <v>Give me a day-by-day sales view for SKU-00022, SKU-00027, SKU-00031 between 2025-01-08 and 2025-01-14, including units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for the whole business. Exclude returned rows.</v>
+        <v>Give me a day-by-day sales view for SKU-00022, SKU-00027, SKU-00031 between 2025-01-08 and 2025-01-14, including units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for the whole business. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L4" t="str">
         <v>query_log_rollup_02</v>
@@ -723,7 +726,7 @@
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-01-08')
     AND business_date &lt;= DATE('2025-01-14')
 ),
@@ -746,13 +749,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-01-08')
     AND business_date &lt;= DATE('2025-01-14')
     AND item_sku IN ('SKU-00022', 'SKU-00027', 'SKU-00031')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -779,7 +783,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K5" t="str">
-        <v>Give me the daily SKU trend for SKU-00022, SKU-00027, SKU-00031 between 2025-01-08 and 2025-01-14, and backfill missing dates with zeroes when nothing sold. Exclude returned rows.</v>
+        <v>Give me the daily SKU trend for SKU-00022, SKU-00027, SKU-00031 between 2025-01-08 and 2025-01-14, and backfill missing dates with zeroes when nothing sold. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L5" t="str">
         <v>query_log_zero_fill_02</v>
@@ -826,13 +830,14 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
 WHERE business_date &gt;= DATE('2025-01-15')
   AND business_date &lt;= DATE('2025-01-21')
   AND item_sku IN ('SKU-00044', 'SKU-00048', 'SKU-00053')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
 GROUP BY item_sku, business_date
 ORDER BY item_sku, business_date;</v>
       </c>
@@ -849,7 +854,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K6" t="str">
-        <v>I want the daily SKU totals for SKU-00044, SKU-00048, SKU-00053 over 2025-01-15 to 2025-01-21 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) rolled up across every store. Exclude returned rows.</v>
+        <v>I want the daily SKU totals for SKU-00044, SKU-00048, SKU-00053 over 2025-01-15 to 2025-01-21 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) rolled up across every store. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L6" t="str">
         <v>query_log_rollup_03</v>
@@ -858,7 +863,7 @@
         <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
       </c>
       <c r="N6">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O6" t="str">
         <v>dataset_retailer_transactions_demo</v>
@@ -897,7 +902,7 @@
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-01-15')
     AND business_date &lt;= DATE('2025-01-21')
 ),
@@ -920,13 +925,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-01-15')
     AND business_date &lt;= DATE('2025-01-21')
     AND item_sku IN ('SKU-00044', 'SKU-00048', 'SKU-00053')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -953,7 +959,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K7" t="str">
-        <v>I need a complete SKU-by-day series for SKU-00044, SKU-00048, SKU-00053 from 2025-01-15 to 2025-01-21, with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) set to 0 on no-sale days. Exclude returned rows.</v>
+        <v>I need a complete SKU-by-day series for SKU-00044, SKU-00048, SKU-00053 from 2025-01-15 to 2025-01-21, with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) set to 0 on no-sale days. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L7" t="str">
         <v>query_log_zero_fill_03</v>
@@ -1000,13 +1006,14 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
 WHERE business_date &gt;= DATE('2025-01-22')
   AND business_date &lt;= DATE('2025-01-31')
   AND item_sku IN ('SKU-00061', 'SKU-00064', 'SKU-00069')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
 GROUP BY item_sku, business_date
 ORDER BY item_sku, business_date;</v>
       </c>
@@ -1023,7 +1030,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K8" t="str">
-        <v>Can you break out daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for SKU-00061, SKU-00064, SKU-00069 from 2025-01-22 through 2025-01-31, summed across all stores? Exclude returned rows.</v>
+        <v>Can you break out daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for SKU-00061, SKU-00064, SKU-00069 from 2025-01-22 through 2025-01-31, summed across all stores? Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L8" t="str">
         <v>query_log_rollup_04</v>
@@ -1032,7 +1039,7 @@
         <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
       </c>
       <c r="N8">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="O8" t="str">
         <v>dataset_retailer_transactions_demo</v>
@@ -1071,7 +1078,7 @@
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-01-22')
     AND business_date &lt;= DATE('2025-01-31')
 ),
@@ -1094,13 +1101,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-01-22')
     AND business_date &lt;= DATE('2025-01-31')
     AND item_sku IN ('SKU-00061', 'SKU-00064', 'SKU-00069')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -1127,7 +1135,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K9" t="str">
-        <v>Return the daily all-store metrics for SKU-00061, SKU-00064, SKU-00069 over 2025-01-22 to 2025-01-31, making sure dates with no sales still appear as zeroes. Exclude returned rows.</v>
+        <v>Return the daily all-store metrics for SKU-00061, SKU-00064, SKU-00069 over 2025-01-22 to 2025-01-31, making sure dates with no sales still appear as zeroes. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L9" t="str">
         <v>query_log_zero_fill_04</v>
@@ -1174,13 +1182,14 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
 WHERE business_date &gt;= DATE('2025-02-01')
   AND business_date &lt;= DATE('2025-02-07')
   AND item_sku IN ('SKU-00078', 'SKU-00082', 'SKU-00086')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
 GROUP BY item_sku, business_date
 ORDER BY item_sku, business_date;</v>
       </c>
@@ -1197,7 +1206,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K10" t="str">
-        <v>Pull a daily all-store SKU summary for SKU-00078, SKU-00082, SKU-00086 between 2025-02-01 and 2025-02-07 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT). Exclude returned rows.</v>
+        <v>Pull a daily all-store SKU summary for SKU-00078, SKU-00082, SKU-00086 between 2025-02-01 and 2025-02-07 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT). Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L10" t="str">
         <v>query_log_rollup_05</v>
@@ -1206,7 +1215,7 @@
         <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
       </c>
       <c r="N10">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O10" t="str">
         <v>dataset_retailer_transactions_demo</v>
@@ -1245,7 +1254,7 @@
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-02-01')
     AND business_date &lt;= DATE('2025-02-07')
 ),
@@ -1268,13 +1277,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-02-01')
     AND business_date &lt;= DATE('2025-02-07')
     AND item_sku IN ('SKU-00078', 'SKU-00082', 'SKU-00086')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -1301,7 +1311,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K11" t="str">
-        <v>Build the same daily rollup for SKU-00078, SKU-00082, SKU-00086 from 2025-02-01 through 2025-02-07, but don’t drop empty days; fill them with 0s instead. Exclude returned rows.</v>
+        <v>Build the same daily rollup for SKU-00078, SKU-00082, SKU-00086 from 2025-02-01 through 2025-02-07, but don’t drop empty days; fill them with 0s instead. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L11" t="str">
         <v>query_log_zero_fill_05</v>
@@ -1348,13 +1358,14 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
 WHERE business_date &gt;= DATE('2025-02-08')
   AND business_date &lt;= DATE('2025-02-14')
   AND item_sku IN ('SKU-00094', 'SKU-00099', 'SKU-00104')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
 GROUP BY item_sku, business_date
 ORDER BY item_sku, business_date;</v>
       </c>
@@ -1371,7 +1382,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K12" t="str">
-        <v>Show daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) across all stores for SKU-00094, SKU-00099, SKU-00104 from 2025-02-08 to 2025-02-14. Exclude returned rows.</v>
+        <v>Show daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) across all stores for SKU-00094, SKU-00099, SKU-00104 from 2025-02-08 to 2025-02-14. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L12" t="str">
         <v>query_log_rollup_06</v>
@@ -1380,7 +1391,7 @@
         <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
       </c>
       <c r="N12">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="O12" t="str">
         <v>dataset_retailer_transactions_demo</v>
@@ -1419,7 +1430,7 @@
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-02-08')
     AND business_date &lt;= DATE('2025-02-14')
 ),
@@ -1442,13 +1453,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-02-08')
     AND business_date &lt;= DATE('2025-02-14')
     AND item_sku IN ('SKU-00094', 'SKU-00099', 'SKU-00104')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -1475,7 +1487,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K13" t="str">
-        <v>Show the same daily SKU metrics across all stores for SKU-00094, SKU-00099, SKU-00104 from 2025-02-08 to 2025-02-14, but include zero rows for days with no sales. Exclude returned rows.</v>
+        <v>Show the same daily SKU metrics across all stores for SKU-00094, SKU-00099, SKU-00104 from 2025-02-08 to 2025-02-14, but include zero rows for days with no sales. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L13" t="str">
         <v>query_log_zero_fill_06</v>
@@ -1522,13 +1534,14 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
 WHERE business_date &gt;= DATE('2025-02-15')
   AND business_date &lt;= DATE('2025-02-21')
   AND item_sku IN ('SKU-00111', 'SKU-00115', 'SKU-00119')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
 GROUP BY item_sku, business_date
 ORDER BY item_sku, business_date;</v>
       </c>
@@ -1545,7 +1558,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K14" t="str">
-        <v>Give me a day-by-day sales view for SKU-00111, SKU-00115, SKU-00119 between 2025-02-15 and 2025-02-21, including units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for the whole business. Exclude returned rows.</v>
+        <v>Give me a day-by-day sales view for SKU-00111, SKU-00115, SKU-00119 between 2025-02-15 and 2025-02-21, including units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for the whole business. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L14" t="str">
         <v>query_log_rollup_07</v>
@@ -1554,7 +1567,7 @@
         <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
       </c>
       <c r="N14">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O14" t="str">
         <v>dataset_retailer_transactions_demo</v>
@@ -1593,7 +1606,7 @@
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-02-15')
     AND business_date &lt;= DATE('2025-02-21')
 ),
@@ -1616,13 +1629,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-02-15')
     AND business_date &lt;= DATE('2025-02-21')
     AND item_sku IN ('SKU-00111', 'SKU-00115', 'SKU-00119')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -1649,7 +1663,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K15" t="str">
-        <v>Give me the daily SKU trend for SKU-00111, SKU-00115, SKU-00119 between 2025-02-15 and 2025-02-21, and backfill missing dates with zeroes when nothing sold. Exclude returned rows.</v>
+        <v>Give me the daily SKU trend for SKU-00111, SKU-00115, SKU-00119 between 2025-02-15 and 2025-02-21, and backfill missing dates with zeroes when nothing sold. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L15" t="str">
         <v>query_log_zero_fill_07</v>
@@ -1696,13 +1710,14 @@
         <v xml:space="preserve">SELECT
   item_sku,
   business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
 WHERE business_date &gt;= DATE('2025-02-22')
   AND business_date &lt;= DATE('2025-02-28')
   AND item_sku IN ('SKU-00127', 'SKU-00132', 'SKU-00137')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
 GROUP BY item_sku, business_date
 ORDER BY item_sku, business_date;</v>
       </c>
@@ -1719,7 +1734,7 @@
         <v>sku_daily_rollup</v>
       </c>
       <c r="K16" t="str">
-        <v>I want the daily SKU totals for SKU-00127, SKU-00132, SKU-00137 over 2025-02-22 to 2025-02-28 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) rolled up across every store. Exclude returned rows.</v>
+        <v>I want the daily SKU totals for SKU-00127, SKU-00132, SKU-00137 over 2025-02-22 to 2025-02-28 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) rolled up across every store. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L16" t="str">
         <v>query_log_rollup_08</v>
@@ -1728,7 +1743,7 @@
         <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
       </c>
       <c r="N16">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="O16" t="str">
         <v>dataset_retailer_transactions_demo</v>
@@ -1767,7 +1782,7 @@
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-02-22')
     AND business_date &lt;= DATE('2025-02-28')
 ),
@@ -1790,13 +1805,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-02-22')
     AND business_date &lt;= DATE('2025-02-28')
     AND item_sku IN ('SKU-00127', 'SKU-00132', 'SKU-00137')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -1823,7 +1839,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K17" t="str">
-        <v>I need a complete SKU-by-day series for SKU-00127, SKU-00132, SKU-00137 from 2025-02-22 to 2025-02-28, with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) set to 0 on no-sale days. Exclude returned rows.</v>
+        <v>I need a complete SKU-by-day series for SKU-00127, SKU-00132, SKU-00137 from 2025-02-22 to 2025-02-28, with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) set to 0 on no-sale days. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L17" t="str">
         <v>query_log_zero_fill_08</v>
@@ -1867,81 +1883,11 @@
         <v>2026-03-18T11:12:01.800Z</v>
       </c>
       <c r="F18" t="str" xml:space="preserve">
-        <v xml:space="preserve">SELECT
-  item_sku,
-  business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
-WHERE business_date &gt;= DATE('2025-03-01')
-  AND business_date &lt;= DATE('2025-03-15')
-  AND item_sku IN ('SKU-00146', 'SKU-00152', 'SKU-00158')
-GROUP BY item_sku, business_date
-ORDER BY item_sku, business_date;</v>
-      </c>
-      <c r="G18" t="str">
-        <v>2026-03-18T11:12:01.760Z</v>
-      </c>
-      <c r="H18">
-        <v>1760</v>
-      </c>
-      <c r="I18" t="str">
-        <v>2026-03-18T11:12:00.000Z</v>
-      </c>
-      <c r="J18" t="str">
-        <v>sku_daily_rollup</v>
-      </c>
-      <c r="K18" t="str">
-        <v>Can you break out daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for SKU-00146, SKU-00152, SKU-00158 from 2025-03-01 through 2025-03-15, summed across all stores? Exclude returned rows.</v>
-      </c>
-      <c r="L18" t="str">
-        <v>query_log_rollup_09</v>
-      </c>
-      <c r="M18" t="str">
-        <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
-      </c>
-      <c r="N18">
-        <v>40</v>
-      </c>
-      <c r="O18" t="str">
-        <v>dataset_retailer_transactions_demo</v>
-      </c>
-      <c r="P18" t="str">
-        <v>succeeded</v>
-      </c>
-      <c r="Q18" t="str">
-        <v>Aggregates units sold, revenue, and cost by SKU and business day across all stores.</v>
-      </c>
-      <c r="R18">
-        <v>2244</v>
-      </c>
-      <c r="S18" t="str">
-        <v>[]</v>
-      </c>
-    </row>
-    <row r="19" xml:space="preserve">
-      <c r="A19" t="str">
-        <v>clean_retailer_transactions_demo_v1</v>
-      </c>
-      <c r="B19" t="str">
-        <v/>
-      </c>
-      <c r="C19" t="str">
-        <v>2026-03-18T11:16:03.082Z</v>
-      </c>
-      <c r="D19">
-        <v>882</v>
-      </c>
-      <c r="E19" t="str">
-        <v>2026-03-18T11:16:02.200Z</v>
-      </c>
-      <c r="F19" t="str" xml:space="preserve">
         <v xml:space="preserve">WITH date_spine AS (
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-03-01')
     AND business_date &lt;= DATE('2025-03-15')
 ),
@@ -1964,13 +1910,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
   WHERE business_date &gt;= DATE('2025-03-01')
     AND business_date &lt;= DATE('2025-03-15')
     AND item_sku IN ('SKU-00146', 'SKU-00152', 'SKU-00158')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -1984,146 +1931,76 @@
   ON daily_sales.sku_day_key = sku_day_spine.sku_day_key
 ORDER BY sku_day_spine.item_sku, sku_day_spine.business_date;</v>
       </c>
-      <c r="G19" t="str">
-        <v>2026-03-18T11:16:02.160Z</v>
-      </c>
-      <c r="H19">
-        <v>2160</v>
-      </c>
-      <c r="I19" t="str">
-        <v>2026-03-18T11:16:00.000Z</v>
-      </c>
-      <c r="J19" t="str">
-        <v>sku_daily_rollup_zero_fill</v>
-      </c>
-      <c r="K19" t="str">
-        <v>Return the daily all-store metrics for SKU-00146, SKU-00152, SKU-00158 over 2025-03-01 to 2025-03-15, making sure dates with no sales still appear as zeroes. Exclude returned rows.</v>
-      </c>
-      <c r="L19" t="str">
-        <v>query_log_zero_fill_09</v>
-      </c>
-      <c r="M19" t="str">
+      <c r="G18" t="str">
+        <v>2026-03-18T11:12:01.760Z</v>
+      </c>
+      <c r="H18">
+        <v>1760</v>
+      </c>
+      <c r="I18" t="str">
+        <v>2026-03-18T11:12:00.000Z</v>
+      </c>
+      <c r="J18" t="str">
+        <v>sku_daily_rollup</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Can you break out daily units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT) for SKU-00146, SKU-00152, SKU-00158 from 2025-03-01 through 2025-03-15, summed across all stores? Exclude returned rows from the metrics, include every business_date in the range for every SKU, and set units_sold, revenue_incl_vat, and cost_ex_vat to 0 when a day has no non-return sales (including return-only days). Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
+      </c>
+      <c r="L18" t="str">
+        <v>query_log_rollup_09</v>
+      </c>
+      <c r="M18" t="str">
         <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
       </c>
-      <c r="N19">
+      <c r="N18">
         <v>45</v>
       </c>
-      <c r="O19" t="str">
+      <c r="O18" t="str">
         <v>dataset_retailer_transactions_demo</v>
       </c>
-      <c r="P19" t="str">
+      <c r="P18" t="str">
         <v>succeeded</v>
       </c>
-      <c r="Q19" t="str">
-        <v>Builds a complete SKU-by-day series and fills missing sales days with zeroes.</v>
-      </c>
-      <c r="R19">
-        <v>3042</v>
-      </c>
-      <c r="S19" t="str">
+      <c r="Q18" t="str">
+        <v>Aggregates units sold, revenue, and cost by SKU and business day across all stores.</v>
+      </c>
+      <c r="R18">
+        <v>2244</v>
+      </c>
+      <c r="S18" t="str">
         <v>[]</v>
       </c>
     </row>
-    <row r="20" xml:space="preserve">
-      <c r="A20" t="str">
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
         <v>clean_retailer_transactions_demo_v1</v>
       </c>
-      <c r="B20" t="str">
+      <c r="B19" t="str">
         <v/>
       </c>
-      <c r="C20" t="str">
-        <v>2026-03-18T11:21:02.382Z</v>
-      </c>
-      <c r="D20">
-        <v>512</v>
-      </c>
-      <c r="E20" t="str">
-        <v>2026-03-18T11:21:01.870Z</v>
-      </c>
-      <c r="F20" t="str" xml:space="preserve">
-        <v xml:space="preserve">SELECT
-  item_sku,
-  business_date,
-  SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-  SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-  SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-FROM clean_transactions
-WHERE business_date &gt;= DATE('2025-03-16')
-  AND business_date &lt;= DATE('2025-03-31')
-  AND item_sku IN ('SKU-00163', 'SKU-00169', 'SKU-00175')
-GROUP BY item_sku, business_date
-ORDER BY item_sku, business_date;</v>
-      </c>
-      <c r="G20" t="str">
-        <v>2026-03-18T11:21:01.830Z</v>
-      </c>
-      <c r="H20">
-        <v>1830</v>
-      </c>
-      <c r="I20" t="str">
-        <v>2026-03-18T11:21:00.000Z</v>
-      </c>
-      <c r="J20" t="str">
-        <v>sku_daily_rollup</v>
-      </c>
-      <c r="K20" t="str">
-        <v>Pull a daily all-store SKU summary for SKU-00163, SKU-00169, SKU-00175 between 2025-03-16 and 2025-03-31 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT). Exclude returned rows.</v>
-      </c>
-      <c r="L20" t="str">
-        <v>query_log_rollup_10</v>
-      </c>
-      <c r="M20" t="str">
-        <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
-      </c>
-      <c r="N20">
-        <v>42</v>
-      </c>
-      <c r="O20" t="str">
-        <v>dataset_retailer_transactions_demo</v>
-      </c>
-      <c r="P20" t="str">
-        <v>succeeded</v>
-      </c>
-      <c r="Q20" t="str">
-        <v>Aggregates units sold, revenue, and cost by SKU and business day across all stores.</v>
-      </c>
-      <c r="R20">
-        <v>2342</v>
-      </c>
-      <c r="S20" t="str">
-        <v>[]</v>
-      </c>
-    </row>
-    <row r="21" xml:space="preserve">
-      <c r="A21" t="str">
-        <v>clean_retailer_transactions_demo_v1</v>
-      </c>
-      <c r="B21" t="str">
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <v>2026-03-18T11:25:03.201Z</v>
-      </c>
-      <c r="D21">
-        <v>916</v>
-      </c>
-      <c r="E21" t="str">
-        <v>2026-03-18T11:25:02.285Z</v>
-      </c>
-      <c r="F21" t="str" xml:space="preserve">
+      <c r="C19" t="str">
+        <v>2026-03-18T11:16:03.082Z</v>
+      </c>
+      <c r="D19">
+        <v>882</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2026-03-18T11:16:02.200Z</v>
+      </c>
+      <c r="F19" t="str" xml:space="preserve">
         <v xml:space="preserve">WITH date_spine AS (
   SELECT DISTINCT
     business_date,
     1 AS join_key
-  FROM clean_transactions
-  WHERE business_date &gt;= DATE('2025-03-16')
-    AND business_date &lt;= DATE('2025-03-31')
+  FROM transactions
+  WHERE business_date &gt;= DATE('2025-03-01')
+    AND business_date &lt;= DATE('2025-03-15')
 ),
 sku_scope(item_sku, join_key) AS (
   VALUES
-    ('SKU-00163', 1),
-    ('SKU-00169', 1),
-    ('SKU-00175', 1)
+    ('SKU-00146', 1),
+    ('SKU-00152', 1),
+    ('SKU-00158', 1)
 ),
 sku_day_spine AS (
   SELECT
@@ -2138,13 +2015,14 @@
     item_sku,
     business_date,
     item_sku || '|' || business_date AS sku_day_key,
-    SUM(CASE WHEN is_return = 0 THEN units_gross ELSE 0 END) AS units_sold,
-    SUM(CASE WHEN is_return = 0 THEN gross_sales_incl_vat ELSE 0 END) AS revenue_incl_vat,
-    SUM(CASE WHEN is_return = 0 THEN cogs_ex_vat ELSE 0 END) AS cost_ex_vat
-  FROM clean_transactions
-  WHERE business_date &gt;= DATE('2025-03-16')
-    AND business_date &lt;= DATE('2025-03-31')
-    AND item_sku IN ('SKU-00163', 'SKU-00169', 'SKU-00175')
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
+  WHERE business_date &gt;= DATE('2025-03-01')
+    AND business_date &lt;= DATE('2025-03-15')
+    AND item_sku IN ('SKU-00146', 'SKU-00152', 'SKU-00158')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
   GROUP BY item_sku, business_date
 )
 SELECT
@@ -2158,6 +2036,182 @@
   ON daily_sales.sku_day_key = sku_day_spine.sku_day_key
 ORDER BY sku_day_spine.item_sku, sku_day_spine.business_date;</v>
       </c>
+      <c r="G19" t="str">
+        <v>2026-03-18T11:16:02.160Z</v>
+      </c>
+      <c r="H19">
+        <v>2160</v>
+      </c>
+      <c r="I19" t="str">
+        <v>2026-03-18T11:16:00.000Z</v>
+      </c>
+      <c r="J19" t="str">
+        <v>sku_daily_rollup_zero_fill</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Return the daily all-store metrics for SKU-00146, SKU-00152, SKU-00158 over 2025-03-01 to 2025-03-15, making sure dates with no sales still appear as zeroes. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
+      </c>
+      <c r="L19" t="str">
+        <v>query_log_zero_fill_09</v>
+      </c>
+      <c r="M19" t="str">
+        <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
+      </c>
+      <c r="N19">
+        <v>45</v>
+      </c>
+      <c r="O19" t="str">
+        <v>dataset_retailer_transactions_demo</v>
+      </c>
+      <c r="P19" t="str">
+        <v>succeeded</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>Builds a complete SKU-by-day series and fills missing sales days with zeroes.</v>
+      </c>
+      <c r="R19">
+        <v>3042</v>
+      </c>
+      <c r="S19" t="str">
+        <v>[]</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>clean_retailer_transactions_demo_v1</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v>2026-03-18T11:21:02.382Z</v>
+      </c>
+      <c r="D20">
+        <v>512</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2026-03-18T11:21:01.870Z</v>
+      </c>
+      <c r="F20" t="str" xml:space="preserve">
+        <v xml:space="preserve">SELECT
+  item_sku,
+  business_date,
+  SUM(units) AS units_sold,
+  SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+  SUM(cogs_ex_vat) AS cost_ex_vat
+FROM transactions
+WHERE business_date &gt;= DATE('2025-03-16')
+  AND business_date &lt;= DATE('2025-03-31')
+  AND item_sku IN ('SKU-00163', 'SKU-00169', 'SKU-00175')
+  AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
+GROUP BY item_sku, business_date
+ORDER BY item_sku, business_date;</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2026-03-18T11:21:01.830Z</v>
+      </c>
+      <c r="H20">
+        <v>1830</v>
+      </c>
+      <c r="I20" t="str">
+        <v>2026-03-18T11:21:00.000Z</v>
+      </c>
+      <c r="J20" t="str">
+        <v>sku_daily_rollup</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Pull a daily all-store SKU summary for SKU-00163, SKU-00169, SKU-00175 between 2025-03-16 and 2025-03-31 with units sold, gross revenue before returns (incl. VAT), and cost (excl. VAT). Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
+      </c>
+      <c r="L20" t="str">
+        <v>query_log_rollup_10</v>
+      </c>
+      <c r="M20" t="str">
+        <v>["item_sku","business_date","units_sold","revenue_incl_vat","cost_ex_vat"]</v>
+      </c>
+      <c r="N20">
+        <v>27</v>
+      </c>
+      <c r="O20" t="str">
+        <v>dataset_retailer_transactions_demo</v>
+      </c>
+      <c r="P20" t="str">
+        <v>succeeded</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>Aggregates units sold, revenue, and cost by SKU and business day across all stores.</v>
+      </c>
+      <c r="R20">
+        <v>2342</v>
+      </c>
+      <c r="S20" t="str">
+        <v>[]</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>clean_retailer_transactions_demo_v1</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v>2026-03-18T11:25:03.201Z</v>
+      </c>
+      <c r="D21">
+        <v>916</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2026-03-18T11:25:02.285Z</v>
+      </c>
+      <c r="F21" t="str" xml:space="preserve">
+        <v xml:space="preserve">WITH date_spine AS (
+  SELECT DISTINCT
+    business_date,
+    1 AS join_key
+  FROM transactions
+  WHERE business_date &gt;= DATE('2025-03-16')
+    AND business_date &lt;= DATE('2025-03-31')
+),
+sku_scope(item_sku, join_key) AS (
+  VALUES
+    ('SKU-00163', 1),
+    ('SKU-00169', 1),
+    ('SKU-00175', 1)
+),
+sku_day_spine AS (
+  SELECT
+    sku_scope.item_sku,
+    date_spine.business_date,
+    sku_scope.item_sku || '|' || date_spine.business_date AS sku_day_key
+  FROM sku_scope
+  JOIN date_spine ON date_spine.join_key = sku_scope.join_key
+),
+daily_sales AS (
+  SELECT
+    item_sku,
+    business_date,
+    item_sku || '|' || business_date AS sku_day_key,
+    SUM(units) AS units_sold,
+    SUM(gross_sales_incl_vat) AS revenue_incl_vat,
+    SUM(cogs_ex_vat) AS cost_ex_vat
+  FROM transactions
+  WHERE business_date &gt;= DATE('2025-03-16')
+    AND business_date &lt;= DATE('2025-03-31')
+    AND item_sku IN ('SKU-00163', 'SKU-00169', 'SKU-00175')
+    AND LOWER(COALESCE(return_flag, '')) NOT IN ('yes','y','true','1')
+  GROUP BY item_sku, business_date
+)
+SELECT
+  sku_day_spine.item_sku,
+  sku_day_spine.business_date,
+  COALESCE(daily_sales.units_sold, 0) AS units_sold,
+  COALESCE(daily_sales.revenue_incl_vat, 0) AS revenue_incl_vat,
+  COALESCE(daily_sales.cost_ex_vat, 0) AS cost_ex_vat
+FROM sku_day_spine
+LEFT JOIN daily_sales
+  ON daily_sales.sku_day_key = sku_day_spine.sku_day_key
+ORDER BY sku_day_spine.item_sku, sku_day_spine.business_date;</v>
+      </c>
       <c r="G21" t="str">
         <v>2026-03-18T11:25:02.245Z</v>
       </c>
@@ -2171,7 +2225,7 @@
         <v>sku_daily_rollup_zero_fill</v>
       </c>
       <c r="K21" t="str">
-        <v>Build the same daily rollup for SKU-00163, SKU-00169, SKU-00175 from 2025-03-16 through 2025-03-31, but don’t drop empty days; fill them with 0s instead. Exclude returned rows.</v>
+        <v>Build the same daily rollup for SKU-00163, SKU-00169, SKU-00175 from 2025-03-16 through 2025-03-31, but don’t drop empty days; fill them with 0s instead. Exclude returned rows. Return exactly one row per SKU per business_date, and output only these columns in this order: item_sku, business_date, units_sold, revenue_incl_vat, cost_ex_vat.</v>
       </c>
       <c r="L21" t="str">
         <v>query_log_zero_fill_10</v>

</xml_diff>